<commit_message>
RUN-2026-01 G4 pass: taxonomy 1.0, mechanism list 1.0, data dictionary 1.3
All 12 recommendations accepted (GATE-0005). RI-TEC-008 retired, RI-TEC-031
merged into RI-FMW-010, RI-TEC-005 narrowed under R22. Stage 8 started.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/review/RUN-2026-01/G4_taxonomy.xlsx
+++ b/review/RUN-2026-01/G4_taxonomy.xlsx
@@ -7,26 +7,28 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reform issues" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items under each issue" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items fitting no issue" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanisms" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanism proposals" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme doubtful items" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Second-pass check" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alpha lessons" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions needed" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reform issues" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items under each issue" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items fitting no issue" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanisms" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanism proposals" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme doubtful items" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Second-pass check" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alpha lessons" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reform issues'!$A$1:$Q$49</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Items under each issue'!$A$1:$G$236</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Items fitting no issue'!$A$1:$D$138</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Mechanisms'!$A$1:$H$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Mechanism proposals'!$A$1:$G$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Theme doubtful items'!$A$1:$E$293</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Second-pass check'!$A$1:$C$52</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Alpha lessons'!$A$1:$S$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Validation'!$A$1:$A$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Decisions needed'!$A$1:$G$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Reform issues'!$A$1:$S$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Items under each issue'!$A$1:$G$236</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Items fitting no issue'!$A$1:$D$138</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Mechanisms'!$A$1:$H$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Mechanism proposals'!$A$1:$G$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Theme doubtful items'!$A$1:$E$293</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Second-pass check'!$A$1:$C$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Alpha lessons'!$A$1:$S$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Validation'!$A$1:$A$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +445,551 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q49"/>
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="56" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>decision_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>decision_needed</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>what_the_files_show</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>agent_recommendation</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>affects</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>reviewer_decision</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>reviewer_comment</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>G4-D01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Approve the area codes FMW (Chapter 2) and TEC (technology and AI).</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>The codes were left open at G0 (decision log and run record). All 48 draft issues use them, and the labels are country-neutral.</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Approve FMW and TEC.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>All issues</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>accept_recommendation</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Sofia, 30 Oct 2026, GATE-0005</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>G4-D02</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Keep or retire RI-TEC-008 (electronic public consultation platform).</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>It has 12 EU requirement items and no recommendation. Procedure P2 requires a theme issue to rest on at least one in-scope recommendation that meets the materiality test, so it fails as drafted. Its drafter also noted that technology is the channel, not the problem.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Retire it (status retired; the ID stays). Its 12 items then fit no issue.</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>RI-TEC-008</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>accept_recommendation</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Sofia, 30 Oct 2026, GATE-0005</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>G4-D03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Resolve the overlap between RI-TEC-031 and the Chapter 2 issues.</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>All 13 items under RI-TEC-031 are also mapped to Chapter 2 issues (RI-FMW-004; -005; -008 to -011), so it adds no evidence of its own. RI-FMW-005 and RI-FMW-010 already carry the technology theme tags.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Merge RI-TEC-031 into RI-FMW-010 (merged_into); EURES IT items stay under RI-FMW-005.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>RI-TEC-031; RI-FMW-005; RI-FMW-010</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>accept_recommendation</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Sofia, 30 Oct 2026, GATE-0005</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>G4-D04</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Narrow RI-TEC-005 (tax IT and e-services) to fit decision R22.</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>At G3, tax IT upgrades were set as out by default unless the claim concerns an EU connection or a service the public uses online. Most of the 16 items pair the back-office integrated IT tax system with e-services in one sentence or list. The stand-alone Integrated Tax Information System sentences were left out of the 2024 and 2025 reports, so the issue currently reads wider than the extraction.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Narrow the label and definition to taxpayer e-services, and treat the integrated IT tax system as out of the issue except where a quote also covers e-services. Keep the 14 recommendations mapped.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>RI-TEC-005</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>accept_recommendation</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Sofia, 30 Oct 2026, GATE-0005</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>G4-D05</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Decide whether RI-TEC-003 (digital public services) is too broad.</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>It is the largest issue: 119 items from 24 sources, of which 52 are recommendations. A keyword count suggests mostly general e-services (about 54) and business or licensing services (about 39). It may fail the granularity test.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Approve as one issue for version 1.0 and test it at G5 classification. Split only if items cannot be assigned consistently: splitting now would mean remapping without evidence that it is needed.</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>RI-TEC-003</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>accept_recommendation</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Sofia, 30 Oct 2026, GATE-0005</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>G4-D06</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Keep RI-TEC-001 (artificial intelligence) as a separate issue on a thin EU base.</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Two EU recommendation items (MKD-EU-2025-001-0149; MKD-EU-2026-005-0002). A keyword check of all EU text found no missed North Macedonia requirement on AI; the AI law conditions in MKD-EU-2024-007 are Serbia's (page 60). One of the two items only encourages outreach around an AI Factory Antenna, so the base is effectively one firm recommendation.</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Keep it: AI is named in the run scope, and thin EU coverage is itself a finding (ALN-0018). National evidence comes at stage 8.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>RI-TEC-001</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>accept_recommendation</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Sofia, 30 Oct 2026, GATE-0005</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>G4-D07</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Keep or merge the small Chapter 2 issues RI-FMW-011 (EHIC) and RI-FMW-012 (supplementary pensions).</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>RI-FMW-011 has 7 items and is flagged as a merge candidate with RI-FMW-008. RI-FMW-012 has 7 items and one recommendation from one source.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Keep both. EHIC is named in the run scope and supplementary pensions are a distinct acquis topic; neither needs to reach the priority list to stay in the taxonomy.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>RI-FMW-008; RI-FMW-011; RI-FMW-012</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>accept_recommendation</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Sofia, 30 Oct 2026, GATE-0005</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>G4-D08</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Confirm the sector issues on the R12 and R22 boundary.</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>RI-TEC-006 (procurement), -007 (services and professions), -009 (eHealth), -010 (justice), -029 (customs), -030 (justice and home affairs systems) and -032 (other EU systems) sit on the boundary. RI-TEC-010 has 7 recommendations but only 2 not flagged theme_doubtful.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Keep six as online public services or EU connections, which R12 and R22 let in. Keep RI-TEC-010 provisionally and recheck it at G5, because court IT may be back-office under R22.</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>RI-TEC-006; -007; -009; -010; -029; -030; -032</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>accept_recommendation</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Sofia, 30 Oct 2026, GATE-0005</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>G4-D09</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Decide how to handle the flagged doubtful and unmapped items.</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>292 items carry theme_doubtful (288 EU; 4 from non-EU sample sources); 63 are mapped to an issue. 137 EU requirement items fit no issue: mainly chapter-level ratings or doubtful items, plus 5 others that name no specific problem or are chain items. Row-by-row review would be heavy.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Decide by group, not row: accept the unmapped list as it stands, and leave doubtful items flagged until classification, when the materiality test is applied per item. No new issue for domain name registry governance (7 items).</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Theme doubtful items and Items fitting no issue sheets</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>accept_recommendation</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Sofia, 30 Oct 2026, GATE-0005</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>G4-D10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Approve the mechanism list changes.</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Proposals are on the Mechanism proposals sheet: rewordings of MEC-01; -03; -07; -08; -09 and two additions, implementation gap (NEW-01) and low uptake of existing systems (MEC-11). MEC-01 and MEC-03 each have two proposals, one from each drafter. MEC-02 has a blank version field.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Combine the paired rewordings of MEC-01 and MEC-03; accept the other rewordings; add both new mechanisms, as MEC-11 (low uptake) and MEC-12 (implementation gap). Record the list as version 1.0, which also fills the MEC-02 gap.</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>taxonomy/mechanisms.csv</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>accept_recommendation</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Sofia, 30 Oct 2026, GATE-0005</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>G4-D11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Decide how to record issues that span clusters.</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>11 technology issues have a blank cluster because their chapters span clusters, and RI-TEC-004 also has no chapter because its items name none. The data dictionary describes cluster as a cluster number and does not cover this case.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Allow a blank cluster to mean cross-cluster and a blank chapter to mean no chapter stated; record this in the data dictionary with a version change.</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>schemas/data_dictionary.md; 11 RI-TEC issues</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>accept_recommendation</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Sofia, 30 Oct 2026, GATE-0005</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>G4-D12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Decide on the alpha lessons raised at this gate.</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>ALN-0018, ALN-0019 and ALN-0020 are open on the Alpha lessons sheet.</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Accept all three.</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>runs/RUN-2026-01/alpha_learning_log.csv</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>accept_recommendation</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Sofia, 30 Oct 2026, GATE-0005</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G13"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="70" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>validate_data output</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>validate_data 1.2.0: 57 evidence file(s), 2138 item(s), 402 CSV row(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>0 error(s), 0 warning(s)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:A3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -461,8 +1007,10 @@
     <col width="16" customWidth="1" min="13" max="13"/>
     <col width="70" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="15" max="15"/>
-    <col width="19" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="17" customWidth="1" min="16" max="16"/>
+    <col width="36" customWidth="1" min="17" max="17"/>
+    <col width="19" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -543,10 +1091,20 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>recommendations</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>recommendations not theme_doubtful</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
           <t>reviewer_decision</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>reviewer_comment</t>
         </is>
@@ -616,8 +1174,18 @@
           <t>26</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr"/>
-      <c r="Q2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr"/>
+      <c r="S2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -683,8 +1251,18 @@
           <t>12</t>
         </is>
       </c>
-      <c r="P3" s="2" t="inlineStr"/>
-      <c r="Q3" s="2" t="inlineStr"/>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr"/>
+      <c r="S3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -750,8 +1328,18 @@
           <t>12</t>
         </is>
       </c>
-      <c r="P4" s="2" t="inlineStr"/>
-      <c r="Q4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr"/>
+      <c r="S4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -817,8 +1405,18 @@
           <t>14</t>
         </is>
       </c>
-      <c r="P5" s="2" t="inlineStr"/>
-      <c r="Q5" s="2" t="inlineStr"/>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="inlineStr"/>
+      <c r="S5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -888,8 +1486,18 @@
           <t>14</t>
         </is>
       </c>
-      <c r="P6" s="2" t="inlineStr"/>
-      <c r="Q6" s="2" t="inlineStr"/>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr"/>
+      <c r="S6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -955,8 +1563,18 @@
           <t>5</t>
         </is>
       </c>
-      <c r="P7" s="2" t="inlineStr"/>
-      <c r="Q7" s="2" t="inlineStr"/>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="R7" s="2" t="inlineStr"/>
+      <c r="S7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1022,8 +1640,18 @@
           <t>3</t>
         </is>
       </c>
-      <c r="P8" s="2" t="inlineStr"/>
-      <c r="Q8" s="2" t="inlineStr"/>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="R8" s="2" t="inlineStr"/>
+      <c r="S8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1089,8 +1717,18 @@
           <t>19</t>
         </is>
       </c>
-      <c r="P9" s="2" t="inlineStr"/>
-      <c r="Q9" s="2" t="inlineStr"/>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="R9" s="2" t="inlineStr"/>
+      <c r="S9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1152,8 +1790,18 @@
           <t>15</t>
         </is>
       </c>
-      <c r="P10" s="2" t="inlineStr"/>
-      <c r="Q10" s="2" t="inlineStr"/>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="R10" s="2" t="inlineStr"/>
+      <c r="S10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1223,8 +1871,18 @@
           <t>6</t>
         </is>
       </c>
-      <c r="P11" s="2" t="inlineStr"/>
-      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1290,8 +1948,18 @@
           <t>7</t>
         </is>
       </c>
-      <c r="P12" s="2" t="inlineStr"/>
-      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1357,8 +2025,18 @@
           <t>7</t>
         </is>
       </c>
-      <c r="P13" s="2" t="inlineStr"/>
-      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1424,8 +2102,18 @@
           <t>13</t>
         </is>
       </c>
-      <c r="P14" s="2" t="inlineStr"/>
-      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1495,8 +2183,18 @@
           <t>2</t>
         </is>
       </c>
-      <c r="P15" s="2" t="inlineStr"/>
-      <c r="Q15" s="2" t="inlineStr"/>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1566,8 +2264,18 @@
           <t>41</t>
         </is>
       </c>
-      <c r="P16" s="2" t="inlineStr"/>
-      <c r="Q16" s="2" t="inlineStr"/>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="R16" s="2" t="inlineStr"/>
+      <c r="S16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1637,8 +2345,18 @@
           <t>119</t>
         </is>
       </c>
-      <c r="P17" s="2" t="inlineStr"/>
-      <c r="Q17" s="2" t="inlineStr"/>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="R17" s="2" t="inlineStr"/>
+      <c r="S17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1700,8 +2418,18 @@
           <t>10</t>
         </is>
       </c>
-      <c r="P18" s="2" t="inlineStr"/>
-      <c r="Q18" s="2" t="inlineStr"/>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="Q18" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="R18" s="2" t="inlineStr"/>
+      <c r="S18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1771,8 +2499,18 @@
           <t>16</t>
         </is>
       </c>
-      <c r="P19" s="2" t="inlineStr"/>
-      <c r="Q19" s="2" t="inlineStr"/>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="Q19" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="R19" s="2" t="inlineStr"/>
+      <c r="S19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1842,8 +2580,18 @@
           <t>22</t>
         </is>
       </c>
-      <c r="P20" s="2" t="inlineStr"/>
-      <c r="Q20" s="2" t="inlineStr"/>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="Q20" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="R20" s="2" t="inlineStr"/>
+      <c r="S20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1913,8 +2661,18 @@
           <t>19</t>
         </is>
       </c>
-      <c r="P21" s="2" t="inlineStr"/>
-      <c r="Q21" s="2" t="inlineStr"/>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="Q21" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="R21" s="2" t="inlineStr"/>
+      <c r="S21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1984,8 +2742,18 @@
           <t>12</t>
         </is>
       </c>
-      <c r="P22" s="2" t="inlineStr"/>
-      <c r="Q22" s="2" t="inlineStr"/>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Q22" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R22" s="2" t="inlineStr"/>
+      <c r="S22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2051,8 +2819,18 @@
           <t>9</t>
         </is>
       </c>
-      <c r="P23" s="2" t="inlineStr"/>
-      <c r="Q23" s="2" t="inlineStr"/>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="Q23" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="R23" s="2" t="inlineStr"/>
+      <c r="S23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2122,8 +2900,18 @@
           <t>10</t>
         </is>
       </c>
-      <c r="P24" s="2" t="inlineStr"/>
-      <c r="Q24" s="2" t="inlineStr"/>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="Q24" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R24" s="2" t="inlineStr"/>
+      <c r="S24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2189,8 +2977,18 @@
           <t>50</t>
         </is>
       </c>
-      <c r="P25" s="2" t="inlineStr"/>
-      <c r="Q25" s="2" t="inlineStr"/>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="Q25" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="R25" s="2" t="inlineStr"/>
+      <c r="S25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2260,8 +3058,18 @@
           <t>24</t>
         </is>
       </c>
-      <c r="P26" s="2" t="inlineStr"/>
-      <c r="Q26" s="2" t="inlineStr"/>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="Q26" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="R26" s="2" t="inlineStr"/>
+      <c r="S26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2331,8 +3139,18 @@
           <t>32</t>
         </is>
       </c>
-      <c r="P27" s="2" t="inlineStr"/>
-      <c r="Q27" s="2" t="inlineStr"/>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="Q27" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="R27" s="2" t="inlineStr"/>
+      <c r="S27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2398,8 +3216,18 @@
           <t>11</t>
         </is>
       </c>
-      <c r="P28" s="2" t="inlineStr"/>
-      <c r="Q28" s="2" t="inlineStr"/>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="Q28" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="R28" s="2" t="inlineStr"/>
+      <c r="S28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2465,8 +3293,18 @@
           <t>24</t>
         </is>
       </c>
-      <c r="P29" s="2" t="inlineStr"/>
-      <c r="Q29" s="2" t="inlineStr"/>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="Q29" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="R29" s="2" t="inlineStr"/>
+      <c r="S29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2532,8 +3370,18 @@
           <t>13</t>
         </is>
       </c>
-      <c r="P30" s="2" t="inlineStr"/>
-      <c r="Q30" s="2" t="inlineStr"/>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="Q30" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="R30" s="2" t="inlineStr"/>
+      <c r="S30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2595,8 +3443,18 @@
           <t>31</t>
         </is>
       </c>
-      <c r="P31" s="2" t="inlineStr"/>
-      <c r="Q31" s="2" t="inlineStr"/>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="Q31" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="R31" s="2" t="inlineStr"/>
+      <c r="S31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2662,8 +3520,18 @@
           <t>9</t>
         </is>
       </c>
-      <c r="P32" s="2" t="inlineStr"/>
-      <c r="Q32" s="2" t="inlineStr"/>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="Q32" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R32" s="2" t="inlineStr"/>
+      <c r="S32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2729,8 +3597,18 @@
           <t>17</t>
         </is>
       </c>
-      <c r="P33" s="2" t="inlineStr"/>
-      <c r="Q33" s="2" t="inlineStr"/>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Q33" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R33" s="2" t="inlineStr"/>
+      <c r="S33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2796,8 +3674,18 @@
           <t>10</t>
         </is>
       </c>
-      <c r="P34" s="2" t="inlineStr"/>
-      <c r="Q34" s="2" t="inlineStr"/>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="Q34" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="R34" s="2" t="inlineStr"/>
+      <c r="S34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2863,8 +3751,18 @@
           <t>10</t>
         </is>
       </c>
-      <c r="P35" s="2" t="inlineStr"/>
-      <c r="Q35" s="2" t="inlineStr"/>
+      <c r="P35" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="Q35" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="R35" s="2" t="inlineStr"/>
+      <c r="S35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2930,8 +3828,18 @@
           <t>40</t>
         </is>
       </c>
-      <c r="P36" s="2" t="inlineStr"/>
-      <c r="Q36" s="2" t="inlineStr"/>
+      <c r="P36" s="2" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="Q36" s="2" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="R36" s="2" t="inlineStr"/>
+      <c r="S36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2993,8 +3901,18 @@
           <t>23</t>
         </is>
       </c>
-      <c r="P37" s="2" t="inlineStr"/>
-      <c r="Q37" s="2" t="inlineStr"/>
+      <c r="P37" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="Q37" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="R37" s="2" t="inlineStr"/>
+      <c r="S37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3060,8 +3978,18 @@
           <t>10</t>
         </is>
       </c>
-      <c r="P38" s="2" t="inlineStr"/>
-      <c r="Q38" s="2" t="inlineStr"/>
+      <c r="P38" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="Q38" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="R38" s="2" t="inlineStr"/>
+      <c r="S38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3127,8 +4055,18 @@
           <t>18</t>
         </is>
       </c>
-      <c r="P39" s="2" t="inlineStr"/>
-      <c r="Q39" s="2" t="inlineStr"/>
+      <c r="P39" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="Q39" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="R39" s="2" t="inlineStr"/>
+      <c r="S39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3194,8 +4132,18 @@
           <t>17</t>
         </is>
       </c>
-      <c r="P40" s="2" t="inlineStr"/>
-      <c r="Q40" s="2" t="inlineStr"/>
+      <c r="P40" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="Q40" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="R40" s="2" t="inlineStr"/>
+      <c r="S40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3265,8 +4213,18 @@
           <t>23</t>
         </is>
       </c>
-      <c r="P41" s="2" t="inlineStr"/>
-      <c r="Q41" s="2" t="inlineStr"/>
+      <c r="P41" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="Q41" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="R41" s="2" t="inlineStr"/>
+      <c r="S41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3332,8 +4290,18 @@
           <t>33</t>
         </is>
       </c>
-      <c r="P42" s="2" t="inlineStr"/>
-      <c r="Q42" s="2" t="inlineStr"/>
+      <c r="P42" s="2" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="Q42" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="R42" s="2" t="inlineStr"/>
+      <c r="S42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3399,8 +4367,18 @@
           <t>26</t>
         </is>
       </c>
-      <c r="P43" s="2" t="inlineStr"/>
-      <c r="Q43" s="2" t="inlineStr"/>
+      <c r="P43" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="Q43" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="R43" s="2" t="inlineStr"/>
+      <c r="S43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3470,8 +4448,18 @@
           <t>12</t>
         </is>
       </c>
-      <c r="P44" s="2" t="inlineStr"/>
-      <c r="Q44" s="2" t="inlineStr"/>
+      <c r="P44" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="Q44" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="R44" s="2" t="inlineStr"/>
+      <c r="S44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3541,8 +4529,18 @@
           <t>13</t>
         </is>
       </c>
-      <c r="P45" s="2" t="inlineStr"/>
-      <c r="Q45" s="2" t="inlineStr"/>
+      <c r="P45" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="Q45" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="R45" s="2" t="inlineStr"/>
+      <c r="S45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3608,8 +4606,18 @@
           <t>24</t>
         </is>
       </c>
-      <c r="P46" s="2" t="inlineStr"/>
-      <c r="Q46" s="2" t="inlineStr"/>
+      <c r="P46" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="Q46" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="R46" s="2" t="inlineStr"/>
+      <c r="S46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3679,8 +4687,18 @@
           <t>38</t>
         </is>
       </c>
-      <c r="P47" s="2" t="inlineStr"/>
-      <c r="Q47" s="2" t="inlineStr"/>
+      <c r="P47" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="Q47" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="R47" s="2" t="inlineStr"/>
+      <c r="S47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3746,8 +4764,18 @@
           <t>15</t>
         </is>
       </c>
-      <c r="P48" s="2" t="inlineStr"/>
-      <c r="Q48" s="2" t="inlineStr"/>
+      <c r="P48" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="Q48" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="R48" s="2" t="inlineStr"/>
+      <c r="S48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3817,16 +4845,26 @@
           <t>13</t>
         </is>
       </c>
-      <c r="P49" s="2" t="inlineStr"/>
-      <c r="Q49" s="2" t="inlineStr"/>
+      <c r="P49" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="Q49" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="R49" s="2" t="inlineStr"/>
+      <c r="S49" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q49"/>
+  <autoFilter ref="A1:S49"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11642,7 +12680,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14699,7 +15737,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -15106,7 +16144,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -15557,7 +16595,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -23490,7 +24528,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -24394,13 +25432,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S20"/>
+  <dimension ref="A1:S21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -24694,7 +25732,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>ALN-0001</t>
+          <t>ALN-0020</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -24704,74 +25742,70 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>pre-G0</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>G0</t>
+          <t>G4</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>workflow</t>
+          <t>taxonomy_matching</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>change_made</t>
+          <t>did_not_work</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Changing the pilot country from Serbia to North Macedonia before G0 required edits to about thirty files because country, chapter, dates, languages and examples were written into the codebooks, procedures and rules.</t>
+          <t>A draft theme issue with no supporting recommendation reached the G4 package, although procedure P2 requires one, because no tool tests this rule and the drafter only hinted at it in a note.</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>codebooks/CB1_project_explanation.md;codebooks/CB3_limits_and_log.md;procedures/P1_setup_and_sources.md;rules/extraction_rules.md</t>
+          <t>RI-TEC-008</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>countries;chapters</t>
+          <t>chapters;clusters;volume</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Every new country or chapter would have needed the same sweep. Keeping run-specific settings in the run record, CLAUDE.md and the limits log makes the method reusable.</t>
+          <t>With more issues, procedural tests on the taxonomy will be missed if they rely on reading each row.</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Keep method documents country-neutral; add a check before each new run that searches the method documents for country, chapter and date terms.</t>
+          <t>Add the test to validate_data.py once the mapping has a permanent home at stage 9; until then show recommendation counts per issue in the package.</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>F2;E5;LIM-0001;LIM-0002;LIM-0003;LIM-0004;LIM-0005;LIM-0006</t>
+          <t>run_notes 2026-10-30;G4-D02</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>implemented</t>
-        </is>
-      </c>
-      <c r="P4" s="2" t="inlineStr">
-        <is>
-          <t>GATE-0001</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr">
         <is>
           <t>agent</t>
@@ -24783,7 +25817,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>ALN-0002</t>
+          <t>ALN-0001</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -24808,22 +25842,22 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>taxonomy_matching</t>
+          <t>workflow</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>methodological_issue</t>
+          <t>change_made</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>A scope combining one chapter with a cross-cutting theme (technology and AI) could not be expressed with chapter and cluster fields alone, so theme tags planned for a later stage had to be brought forward.</t>
+          <t>Changing the pilot country from Serbia to North Macedonia before G0 required edits to about thirty files because country, chapter, dates, languages and examples were written into the codebooks, procedures and rules.</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>taxonomy/themes.csv;schemas/evidence_item.schema.json</t>
+          <t>codebooks/CB1_project_explanation.md;codebooks/CB3_limits_and_log.md;procedures/P1_setup_and_sources.md;rules/extraction_rules.md</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -24833,27 +25867,27 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>chapters;clusters</t>
+          <t>countries;chapters</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Scaling across chapters and clusters will need more cross-cutting themes; the materiality test and scope basis need testing at G3 to G5 before more themes are added.</t>
+          <t>Every new country or chapter would have needed the same sweep. Keeping run-specific settings in the run record, CLAUDE.md and the limits log makes the method reusable.</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Review how well the materiality test and the out_of_scope check work at G3 and G5 before defining further themes.</t>
+          <t>Keep method documents country-neutral; add a check before each new run that searches the method documents for country, chapter and date terms.</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>D5;D6;A6;run_notes 2026-10-29</t>
+          <t>F2;E5;LIM-0001;LIM-0002;LIM-0003;LIM-0004;LIM-0005;LIM-0006</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>accepted</t>
+          <t>implemented</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -24872,7 +25906,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>ALN-0003</t>
+          <t>ALN-0002</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -24887,7 +25921,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>pre-G0</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -24897,52 +25931,52 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>tooling</t>
+          <t>taxonomy_matching</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>technical_issue</t>
+          <t>methodological_issue</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>The helper tools depend on system software (text recognition with Macedonian and Albanian language data, PDF rendering) that was not installed in the working environment and was not recorded anywhere before stage 0.</t>
+          <t>A scope combining one chapter with a cross-cutting theme (technology and AI) could not be expressed with chapter and cluster fields alone, so theme tags planned for a later stage had to be brought forward.</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>tools/requirements.txt;tools/tests/last_report.csv</t>
+          <t>taxonomy/themes.csv;schemas/evidence_item.schema.json</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>countries;languages</t>
+          <t>chapters;clusters</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Each new country or language needs its own text recognition data and a test with a sample in that script before extraction starts.</t>
+          <t>Scaling across chapters and clusters will need more cross-cutting themes; the materiality test and scope basis need testing at G3 to G5 before more themes are added.</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>Keep tools/requirements.txt current; add a scanned sample in each new language to tools/tests/test_tools.py before a new country is added.</t>
+          <t>Review how well the materiality test and the out_of_scope check work at G3 and G5 before defining further themes.</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>run_notes 2026-10-29</t>
+          <t>D5;D6;A6;run_notes 2026-10-29</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>implemented</t>
+          <t>accepted</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -24961,7 +25995,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>ALN-0004</t>
+          <t>ALN-0003</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -24976,32 +26010,32 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>G1</t>
+          <t>G0</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>workflow</t>
+          <t>tooling</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>methodological_issue</t>
+          <t>technical_issue</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>The rule that the freeze date falls just after the annual enlargement package did not match the date set at G0: the 2026 package had not appeared by the freeze date, so the newest annual report in the run is from 2025.</t>
+          <t>The helper tools depend on system software (text recognition with Macedonian and Albanian language data, PDF rendering) that was not installed in the working environment and was not recorded anywhere before stage 0.</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>REQ-001</t>
+          <t>tools/requirements.txt;tools/tests/last_report.csv</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -25011,32 +26045,32 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>countries;volume</t>
+          <t>countries;languages</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Every country shares the same package date, so a freeze date set before the package leaves all countries a year behind; a date set after it must wait for publication.</t>
+          <t>Each new country or language needs its own text recognition data and a test with a sample in that script before extraction starts.</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>At G0, check whether the year's package has been published before fixing the freeze date, and record which annual report is the latest in scope.</t>
+          <t>Keep tools/requirements.txt current; add a scanned sample in each new language to tools/tests/test_tools.py before a new country is added.</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>A3;A7;GATE-0001;run_notes 2026-10-29</t>
+          <t>run_notes 2026-10-29</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>accepted</t>
+          <t>implemented</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>GATE-0002</t>
+          <t>GATE-0001</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr">
@@ -25050,7 +26084,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>ALN-0005</t>
+          <t>ALN-0004</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -25075,47 +26109,47 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>sources</t>
+          <t>workflow</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>limitation_found</t>
+          <t>methodological_issue</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>A cross-cutting theme makes the whole of each annual report and the screening reports for all clusters relevant, so the EU source base is much larger than for a single chapter.</t>
+          <t>The rule that the freeze date falls just after the annual enlargement package did not match the date set at G0: the 2026 package had not appeared by the freeze date, so the newest annual report in the run is from 2025.</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>REQ-001;REQ-004;REQ-005</t>
+          <t>REQ-001</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>chapters;clusters;volume</t>
+          <t>countries;volume</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Workload grows with the number of themes rather than the number of chapters; adding themes will need more extraction effort and a sharper materiality test.</t>
+          <t>Every country shares the same package date, so a freeze date set before the package leaves all countries a year behind; a date set after it must wait for publication.</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>Measure extraction time and the share of theme items found incidental at G3 before adding further themes.</t>
+          <t>At G0, check whether the year's package has been published before fixing the freeze date, and record which annual report is the latest in scope.</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>D6;LIM-0009;run_notes 2026-10-29</t>
+          <t>A3;A7;GATE-0001;run_notes 2026-10-29</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
@@ -25139,7 +26173,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>ALN-0006</t>
+          <t>ALN-0005</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -25154,12 +26188,12 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>G2</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -25174,12 +26208,12 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Major publishers (OECD and SIGMA, UNDP, Council of Europe, some Council and national pages) block automated downloads, so several core sources need manual retrieval by the analyst.</t>
+          <t>A cross-cutting theme makes the whole of each annual report and the screening reports for all clusters relevant, so the EU source base is much larger than for a single chapter.</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>MKD-IO-2024-003;MKD-IO-2024-004;MKD-IO-2024-005;MKD-EU-2023-008;MKD-GOV-2020-003</t>
+          <t>REQ-001;REQ-004;REQ-005</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -25189,22 +26223,22 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>countries;volume</t>
+          <t>chapters;clusters;volume</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Manual retrieval grows with every country added and could become the bottleneck of acquisition.</t>
+          <t>Workload grows with the number of themes rather than the number of chapters; adding themes will need more extraction effort and a sharper materiality test.</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>Plan a manual retrieval step in the procedure, or seek permitted access routes (publisher APIs or bulk downloads) before scaling.</t>
+          <t>Measure extraction time and the share of theme items found incidental at G3 before adding further themes.</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>run_notes 2026-10-29;REQ-024;REQ-025</t>
+          <t>D6;LIM-0009;run_notes 2026-10-29</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
@@ -25214,7 +26248,7 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>GATE-0003</t>
+          <t>GATE-0002</t>
         </is>
       </c>
       <c r="Q9" s="2" t="inlineStr">
@@ -25228,7 +26262,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>ALN-0007</t>
+          <t>ALN-0006</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -25263,12 +26297,12 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Almost all national government sources in scope are only in Macedonian (some also in Albanian), so most evidence on the country response will rest on machine translation capped at Medium confidence.</t>
+          <t>Major publishers (OECD and SIGMA, UNDP, Council of Europe, some Council and national pages) block automated downloads, so several core sources need manual retrieval by the analyst.</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>MKD-GOV-2021-001;MKD-GOV-2025-007;MKD-GOV-2024-005</t>
+          <t>MKD-IO-2024-003;MKD-IO-2024-004;MKD-IO-2024-005;MKD-EU-2023-008;MKD-GOV-2020-003</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -25278,22 +26312,22 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>countries;languages</t>
+          <t>countries;volume</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Every new country brings its own language; without a reviewer who reads it, country-response evidence stays capped at Medium.</t>
+          <t>Manual retrieval grows with every country added and could become the bottleneck of acquisition.</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Before scaling, decide whether to recruit reviewers who read the national languages, and measure at G3 how often machine translation affects extraction.</t>
+          <t>Plan a manual retrieval step in the procedure, or seek permitted access routes (publisher APIs or bulk downloads) before scaling.</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>LIM-0012;A8;run_notes 2026-10-29</t>
+          <t>run_notes 2026-10-29;REQ-024;REQ-025</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
@@ -25317,7 +26351,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>ALN-0008</t>
+          <t>ALN-0007</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -25342,47 +26376,47 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>tooling</t>
+          <t>sources</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>technical_issue</t>
+          <t>limitation_found</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Acquisition relied on an unversioned working script; three recording errors were caught and corrected, which shows the step needs a tested tool.</t>
+          <t>Almost all national government sources in scope are only in Macedonian (some also in Albanian), so most evidence on the country response will rest on machine translation capped at Medium confidence.</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>MKD-GOV-2024-001;MKD-EU-2025-014;MKD-EU-2026-005</t>
+          <t>MKD-GOV-2021-001;MKD-GOV-2025-007;MKD-GOV-2024-005</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>countries;volume</t>
+          <t>countries;languages</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>At larger scale, recording errors in the register would be harder to spot by hand.</t>
+          <t>Every new country brings its own language; without a reviewer who reads it, country-response evidence stays capped at Medium.</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Turn the acquisition script into a tested project tool (download, fingerprint, file, convert, register) before the next run.</t>
+          <t>Before scaling, decide whether to recruit reviewers who read the national languages, and measure at G3 how often machine translation affects extraction.</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>run_notes 2026-10-29</t>
+          <t>LIM-0012;A8;run_notes 2026-10-29</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
@@ -25406,7 +26440,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>ALN-0009</t>
+          <t>ALN-0008</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -25431,22 +26465,22 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>workflow</t>
+          <t>tooling</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>worked</t>
+          <t>technical_issue</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Searching for sources with parallel agents, one per group of families, and checking every URL before download found 99 documents in under an hour.</t>
+          <t>Acquisition relied on an unversioned working script; three recording errors were caught and corrected, which shows the step needs a tested tool.</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>REQ-001;REQ-009;REQ-019</t>
+          <t>MKD-GOV-2024-001;MKD-EU-2025-014;MKD-EU-2026-005</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -25456,17 +26490,17 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>countries;chapters;volume</t>
+          <t>countries;volume</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>The approach can scale to more countries and chapters, provided agent-supplied metadata is checked before registration.</t>
+          <t>At larger scale, recording errors in the register would be harder to spot by hand.</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>Keep the per-family split; add a metadata check against the first page of each document.</t>
+          <t>Turn the acquisition script into a tested project tool (download, fingerprint, file, convert, register) before the next run.</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -25495,7 +26529,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>ALN-0010</t>
+          <t>ALN-0009</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -25510,57 +26544,57 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>G3</t>
+          <t>G2</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>extraction</t>
+          <t>workflow</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>limitation_found</t>
+          <t>worked</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>In the sample, the technology theme produced about two and a half times as many items as Chapter 2 (742 against 288), many of them sector IT systems of doubtful relevance, at about 6 to 7 hours of agent time for 11 sources.</t>
+          <t>Searching for sources with parallel agents, one per group of families, and checking every URL before download found 99 documents in under an hour.</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>MKD-EU-2023-001;MKD-EU-2025-001;MKD-EU-2025-003</t>
+          <t>REQ-001;REQ-009;REQ-019</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>chapters;clusters;volume</t>
+          <t>countries;chapters;volume</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>A cross-cutting theme read across whole reports multiplies extraction volume; adding themes or countries would multiply it again.</t>
+          <t>The approach can scale to more countries and chapters, provided agent-supplied metadata is checked before registration.</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>Tighten the materiality test before full extraction (rule issue R1) and measure the effect on the next sample.</t>
+          <t>Keep the per-family split; add a metadata check against the first page of each document.</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>ALN-0005;LIM-0009;run_notes 2026-10-29</t>
+          <t>run_notes 2026-10-29</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
@@ -25570,7 +26604,7 @@
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>GATE-0004</t>
+          <t>GATE-0003</t>
         </is>
       </c>
       <c r="Q13" s="2" t="inlineStr">
@@ -25584,7 +26618,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>ALN-0011</t>
+          <t>ALN-0010</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -25609,47 +26643,47 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>tooling</t>
+          <t>extraction</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>technical_issue</t>
+          <t>limitation_found</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>The quote check cannot verify quotes that cross a page break because printed page numbers and running headers sit between the pages, so sound items were shortened or dropped.</t>
+          <t>In the sample, the technology theme produced about two and a half times as many items as Chapter 2 (742 against 288), many of them sector IT systems of doubtful relevance, at about 6 to 7 hours of agent time for 11 sources.</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>MKD-EU-2025-001;MKD-EU-2023-001-0005;MKD-EU-2025-003-0018</t>
+          <t>MKD-EU-2023-001;MKD-EU-2025-001;MKD-EU-2025-003</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>volume</t>
+          <t>chapters;clusters;volume</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Longer documents and other publishers' layouts will make this more frequent.</t>
+          <t>A cross-cutting theme read across whole reports multiplies extraction volume; adding themes or countries would multiply it again.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>Teach the quote check to skip page-number and header lines at page boundaries (rule issue R4).</t>
+          <t>Tighten the materiality test before full extraction (rule issue R1) and measure the effect on the next sample.</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>run_notes 2026-10-29</t>
+          <t>ALN-0005;LIM-0009;run_notes 2026-10-29</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
@@ -25673,7 +26707,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>ALN-0012</t>
+          <t>ALN-0011</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -25698,42 +26732,42 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>extraction</t>
+          <t>tooling</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>did_not_work</t>
+          <t>technical_issue</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Parallel extraction agents applied the same rules in different ways where the rules were silent (repeated text, sub-area progress wording, chapter basis), which makes counts and later judgements inconsistent.</t>
+          <t>The quote check cannot verify quotes that cross a page break because printed page numbers and running headers sit between the pages, so sound items were shortened or dropped.</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>MKD-EU-2023-001;MKD-EU-2025-001;MKD-EU-2026-005</t>
+          <t>MKD-EU-2025-001;MKD-EU-2023-001-0005;MKD-EU-2025-003-0018</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>countries;chapters;volume</t>
+          <t>volume</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>The more sources and agents, the more such differences will accumulate unless the rules cover these cases.</t>
+          <t>Longer documents and other publishers' layouts will make this more frequent.</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>Add the clarifications in rule issues R3, R7, R10 and R11 and give every extraction agent the same worked examples.</t>
+          <t>Teach the quote check to skip page-number and header lines at page boundaries (rule issue R4).</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
@@ -25762,7 +26796,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>ALN-0013</t>
+          <t>ALN-0012</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -25777,7 +26811,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -25797,32 +26831,32 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>The automatic quote check confirms that a quote appears at its location but not that it is cut to the claim; three quotes that began too early passed it unnoticed until an agent re-read them.</t>
+          <t>Parallel extraction agents applied the same rules in different ways where the rules were silent (repeated text, sub-area progress wording, chapter basis), which makes counts and later judgements inconsistent.</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>MKD-EU-2023-001-0037;MKD-EU-2023-001-0117;MKD-EU-2023-001-0150</t>
+          <t>MKD-EU-2023-001;MKD-EU-2025-001;MKD-EU-2026-005</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>volume</t>
+          <t>countries;chapters;volume</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>At larger volumes, mis-cut quotes will only be caught by sampling, so they could reach judgements.</t>
+          <t>The more sources and agents, the more such differences will accumulate unless the rules cover these cases.</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>Warn on quotes longer than three sentences and keep quote boundaries in the reviewer checklist (rule issue R18).</t>
+          <t>Add the clarifications in rule issues R3, R7, R10 and R11 and give every extraction agent the same worked examples.</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -25851,7 +26885,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>ALN-0014</t>
+          <t>ALN-0013</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -25881,17 +26915,17 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>worked</t>
+          <t>did_not_work</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Applying analyst decisions R1 to R11 by revising the sample, rather than re-extracting it, took about half an hour per source and cut the sample from 1,054 to 732 items with every quote still verified; it also surfaced the next layer of boundary questions.</t>
+          <t>The automatic quote check confirms that a quote appears at its location but not that it is cut to the claim; three quotes that began too early passed it unnoticed until an agent re-read them.</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>review/RUN-2026-01/sample_0.1b;review/RUN-2026-01/G3_rule_issues.csv</t>
+          <t>MKD-EU-2023-001-0037;MKD-EU-2023-001-0117;MKD-EU-2023-001-0150</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
@@ -25901,17 +26935,17 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>chapters;countries;volume</t>
+          <t>volume</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>Rule refinement in short loops on a fixed sample is cheap, and each loop exposes boundary cases that need a written rule before scaling.</t>
+          <t>At larger volumes, mis-cut quotes will only be caught by sampling, so they could reach judgements.</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>Keep the revise-and-compare loop at G3 for every new chapter or theme, with a fixed sample and a comparison sheet.</t>
+          <t>Warn on quotes longer than three sentences and keep quote boundaries in the reviewer checklist (rule issue R18).</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
@@ -25940,7 +26974,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>ALN-0015</t>
+          <t>ALN-0014</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -25965,42 +26999,42 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>review_gates</t>
+          <t>extraction</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>change_made</t>
+          <t>worked</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>The manual extraction check was reduced to simplified hand-coding of three passages and a stratified sample of 70 items, focused on missed and misclassified items, instead of reviewing every extracted item.</t>
+          <t>Applying analyst decisions R1 to R11 by revising the sample, rather than re-extracting it, took about half an hour per source and cut the sample from 1,054 to 732 items with every quote still verified; it also surfaced the next layer of boundary questions.</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>review/RUN-2026-01/G3_review_sample.xlsx;review/RUN-2026-01/G3_handcoding.xlsx</t>
+          <t>review/RUN-2026-01/sample_0.1b;review/RUN-2026-01/G3_rule_issues.csv</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>countries;chapters;volume</t>
+          <t>chapters;countries;volume</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>Reviewing every item does not scale; a fixed-size stratified sample keeps the analyst workload roughly constant as volume grows.</t>
+          <t>Rule refinement in short loops on a fixed sample is cheap, and each loop exposes boundary cases that need a written rule before scaling.</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>Confirm at G3 whether the sample gave enough confidence; if so, make the stratified sample the standard G3 check in procedure P2.</t>
+          <t>Keep the revise-and-compare loop at G3 for every new chapter or theme, with a fixed sample and a comparison sheet.</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
@@ -26029,7 +27063,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>ALN-0016</t>
+          <t>ALN-0015</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -26059,17 +27093,17 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>worked</t>
+          <t>change_made</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Independent agents (a blind coder and reviewers who took no part in extraction) checked all 725 sample items in under 15 minutes elapsed, recorded verdicts before fixing, and gave usable error rates without analyst time.</t>
+          <t>The manual extraction check was reduced to simplified hand-coding of three passages and a stratified sample of 70 items, focused on missed and misclassified items, instead of reviewing every extracted item.</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>review/RUN-2026-01/g3_qa/g3_metrics.csv</t>
+          <t>review/RUN-2026-01/G3_review_sample.xlsx;review/RUN-2026-01/G3_handcoding.xlsx</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -26084,17 +27118,17 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>Independent agent review scales with volume where human row review cannot; the remaining gap is that no human has checked extraction directly.</t>
+          <t>Reviewing every item does not scale; a fixed-size stratified sample keeps the analyst workload roughly constant as volume grows.</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>Keep agent QA as the standard G3 check; add a small human spot check (about 10 items) when a new country or language is added.</t>
+          <t>Confirm at G3 whether the sample gave enough confidence; if so, make the stratified sample the standard G3 check in procedure P2.</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>E12;run_notes 2026-10-29</t>
+          <t>run_notes 2026-10-29</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
@@ -26118,7 +27152,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>ALN-0017</t>
+          <t>ALN-0016</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -26143,22 +27177,22 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>extraction</t>
+          <t>review_gates</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>did_not_work</t>
+          <t>worked</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>The main extraction weaknesses are missed neighbouring claims (about 14% of in-scope claims, mostly low or medium importance) and quotes that hold two claims; types and references are almost always right.</t>
+          <t>Independent agents (a blind coder and reviewers who took no part in extraction) checked all 725 sample items in under 15 minutes elapsed, recorded verdicts before fixing, and gave usable error rates without analyst time.</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>MKD-EU-2023-001-0208;MKD-EU-2025-001-0205;MKD-GOV-2025-011-0118</t>
+          <t>review/RUN-2026-01/g3_qa/g3_metrics.csv</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -26168,22 +27202,22 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>volume;chapters</t>
+          <t>countries;chapters;volume</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>At full scale, misses concentrate in sections far from the chapter headings; a second screening pass is cheaper than a human check.</t>
+          <t>Independent agent review scales with volume where human row review cannot; the remaining gap is that no human has checked extraction directly.</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>In full extraction, add a second-pass check per source: keyword screen for the theme and a split check for two-claim quotes, run by a different agent.</t>
+          <t>Keep agent QA as the standard G3 check; add a small human spot check (about 10 items) when a new country or language is added.</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>run_notes 2026-10-29</t>
+          <t>E12;run_notes 2026-10-29</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
@@ -26204,47 +27238,97 @@
       <c r="R20" s="2" t="inlineStr"/>
       <c r="S20" s="2" t="inlineStr"/>
     </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>ALN-0017</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>RUN-2026-01</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>did_not_work</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>The main extraction weaknesses are missed neighbouring claims (about 14% of in-scope claims, mostly low or medium importance) and quotes that hold two claims; types and references are almost always right.</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>MKD-EU-2023-001-0208;MKD-EU-2025-001-0205;MKD-GOV-2025-011-0118</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>volume;chapters</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>At full scale, misses concentrate in sections far from the chapter headings; a second screening pass is cheaper than a human check.</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>In full extraction, add a second-pass check per source: keyword screen for the theme and a split check for two-claim quotes, run by a different agent.</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>run_notes 2026-10-29</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>GATE-0004</t>
+        </is>
+      </c>
+      <c r="Q21" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+      <c r="R21" s="2" t="inlineStr"/>
+      <c r="S21" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S20"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="70" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>validate_data output</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>validate_data 1.2.0: 57 evidence file(s), 2138 item(s), 401 CSV row(s)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>0 error(s), 0 warning(s)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:A3"/>
+  <autoFilter ref="A1:S21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>